<commit_message>
Chuan hoa 199 nhom DC (173 goc + 26 moi hom nay) vao file Excel va folder DC Telegram
</commit_message>
<xml_diff>
--- a/Danh_Sach_Chat_ID_Nhom_DC.xlsx
+++ b/Danh_Sach_Chat_ID_Nhom_DC.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DANH_SACH_DC_225" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DANH_SACH_DC_199" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H226"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -461,7 +461,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>THƯ MỤC TELEGRAM</t>
+          <t>TRẠNG THÁI</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -570,7 +570,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -604,7 +604,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -672,7 +672,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -706,7 +706,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -774,7 +774,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -808,7 +808,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -842,7 +842,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -876,7 +876,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -910,7 +910,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -944,7 +944,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -978,7 +978,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
@@ -1033,20 +1033,18 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>-1003847096835</t>
+          <t>-5006156746</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>13</v>
-      </c>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -1067,18 +1065,20 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>-5006156746</t>
+          <t>-1003847096835</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr"/>
+          <t>Supergroup</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr"/>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr"/>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr"/>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr"/>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr"/>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr"/>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr"/>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr"/>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr"/>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr"/>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr"/>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr"/>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr"/>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr"/>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr"/>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr"/>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr"/>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr"/>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr"/>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr"/>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr"/>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr"/>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr"/>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr"/>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr"/>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr"/>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr"/>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr"/>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr"/>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr"/>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr"/>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr"/>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr"/>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr"/>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-5240250375</t>
+          <t>-5169655411</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2977,12 +2977,10 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F74" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr"/>
@@ -3003,7 +3001,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>-5169655411</t>
+          <t>-5240250375</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -3011,10 +3009,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr"/>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr"/>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr"/>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr"/>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr"/>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr"/>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr"/>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr"/>
@@ -3286,7 +3286,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr"/>
@@ -3320,7 +3320,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr"/>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr"/>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr"/>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr"/>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr"/>
@@ -3490,7 +3490,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr"/>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr"/>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr"/>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr"/>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr"/>
@@ -3694,7 +3694,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr"/>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr"/>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr"/>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr"/>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr"/>
@@ -3898,7 +3898,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr"/>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H102" s="3" t="inlineStr"/>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr"/>
@@ -3998,7 +3998,7 @@
       <c r="F104" s="2" t="inlineStr"/>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H104" s="3" t="inlineStr"/>
@@ -4032,7 +4032,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H105" s="3" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H106" s="3" t="inlineStr"/>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H107" s="3" t="inlineStr"/>
@@ -4134,7 +4134,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H108" s="3" t="inlineStr"/>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H109" s="3" t="inlineStr"/>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr"/>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H111" s="3" t="inlineStr"/>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H112" s="3" t="inlineStr"/>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H113" s="3" t="inlineStr"/>
@@ -4338,7 +4338,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr"/>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H115" s="3" t="inlineStr"/>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H116" s="3" t="inlineStr"/>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H117" s="3" t="inlineStr"/>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H118" s="3" t="inlineStr"/>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H119" s="3" t="inlineStr"/>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H120" s="3" t="inlineStr"/>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H121" s="3" t="inlineStr"/>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H122" s="3" t="inlineStr"/>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H123" s="3" t="inlineStr"/>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H124" s="3" t="inlineStr"/>
@@ -4694,25 +4694,25 @@
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>( OFF ) DC - TSO ( Trường Sơn)</t>
+          <t>AV4 - DC (SAV_04-00.03 The Sun Avenue)</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>-1001627610405</t>
+          <t>-4903740099</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F125" s="2" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H125" s="3" t="inlineStr"/>
@@ -4728,12 +4728,12 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>28. TF x DC Long Biên</t>
+          <t>CHR - DC (S01.11 Block A1 Charm Sapphire)</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>-5507549892</t>
+          <t>-4946147649</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -4742,11 +4742,11 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H126" s="3" t="inlineStr"/>
@@ -4762,12 +4762,12 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>AV4 - DC (SAV_04-00.03 The Sun Avenue)</t>
+          <t>CKO - DC (85 Cây Keo)</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>-4903740099</t>
+          <t>-613928063</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -4776,11 +4776,11 @@
         </is>
       </c>
       <c r="F127" s="2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H127" s="3" t="inlineStr"/>
@@ -4796,12 +4796,12 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>BAKERY x DC: HUB BÁNH TƯƠI</t>
+          <t>CLG - DC (64A Cửu Long)</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>-5097435576</t>
+          <t>-4864768952</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -4810,11 +4810,11 @@
         </is>
       </c>
       <c r="F128" s="2" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H128" s="3" t="inlineStr"/>
@@ -4830,12 +4830,12 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>CCDC Khai Trương - Định kỳ</t>
+          <t>CLN - DC</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>-512625105</t>
+          <t>-4870092396</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -4844,11 +4844,11 @@
         </is>
       </c>
       <c r="F129" s="2" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H129" s="3" t="inlineStr"/>
@@ -4864,25 +4864,25 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>CCDC SALE + NCP + SCM</t>
+          <t>CN1 - DC (48 CN1)</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>-1002547246318</t>
+          <t>-868672635</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>354</v>
+        <v>19</v>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H130" s="3" t="inlineStr"/>
@@ -4898,12 +4898,12 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>CHR - DC (S01.11 Block A1 Charm Sapphire)</t>
+          <t>CTH - DC (TMDV Citihome Cát Lái)</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>-4946147649</t>
+          <t>-4117975293</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -4912,11 +4912,11 @@
         </is>
       </c>
       <c r="F131" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H131" s="3" t="inlineStr"/>
@@ -4932,12 +4932,12 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>CKO - DC (85 Cây Keo)</t>
+          <t>D10 - DC (01 Đường Số 10 Tân Kiểng)</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>-613928063</t>
+          <t>-4950196076</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -4946,11 +4946,11 @@
         </is>
       </c>
       <c r="F132" s="2" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H132" s="3" t="inlineStr"/>
@@ -4966,25 +4966,25 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>CLG - DC (64A Cửu Long)</t>
+          <t>DC - 410 PHI (410 Phan Huy Ích)</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>-4864768952</t>
+          <t>-1001878454662</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H133" s="3" t="inlineStr"/>
@@ -5000,12 +5000,12 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>CLN - DC</t>
+          <t>DC - AKR (Akari City)</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>-4870092396</t>
+          <t>-4114032701</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -5014,11 +5014,11 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H134" s="3" t="inlineStr"/>
@@ -5034,25 +5034,25 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>CN1 - DC (48 CN1)</t>
+          <t>DC - BQI (Quận BT) - (Trả tote và rổ)</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>-868672635</t>
+          <t>-1001838756395</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F135" s="2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H135" s="3" t="inlineStr"/>
@@ -5068,12 +5068,12 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>CTH - DC (TMDV Citihome Cát Lái)</t>
+          <t>DC - CLD (Quận 7)-(Trả Thùng xanh)</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>-4117975293</t>
+          <t>-4567680972</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -5082,11 +5082,11 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H136" s="3" t="inlineStr"/>
@@ -5102,25 +5102,25 @@
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>Chuyển kho về Đông Hưng</t>
+          <t>DC - DS3 (Thủ đức)-(Trả Thùng Xanh)</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>-4743767182</t>
+          <t>-1001984727983</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F137" s="2" t="n">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H137" s="3" t="inlineStr"/>
@@ -5136,12 +5136,12 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Cập nhật Thùng/Rổ/Pallet_DC &amp; ST</t>
+          <t>DC - ECG (Eco Green)</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>-832566205</t>
+          <t>-918508542</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -5150,11 +5150,11 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H138" s="3" t="inlineStr"/>
@@ -5170,25 +5170,25 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>D10 - DC (01 Đường Số 10 Tân Kiểng)</t>
+          <t>DC - HTP (571 Huỳnh Tấn Phát)</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>-4950196076</t>
+          <t>-1001695487862</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F139" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H139" s="3" t="inlineStr"/>
@@ -5204,25 +5204,25 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>DC - 410 PHI (410 Phan Huy Ích)</t>
+          <t>DC - KHI (98 Khánh Hội)</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>-1001878454662</t>
+          <t>-4039116350</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H140" s="3" t="inlineStr"/>
@@ -5238,12 +5238,12 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>DC - AKR (Akari City)</t>
+          <t>DC - LTC (97 Lê Thị Chợ)</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>-4114032701</t>
+          <t>-4115684818</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
@@ -5252,11 +5252,11 @@
         </is>
       </c>
       <c r="F141" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H141" s="3" t="inlineStr"/>
@@ -5272,12 +5272,12 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>DC - BQI (Quận BT) - (Trả tote và rổ)</t>
+          <t>DC - LTC (Lê Thị Chợ)</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>-1001838756395</t>
+          <t>-1004451611911</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -5286,11 +5286,11 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H142" s="3" t="inlineStr"/>
@@ -5306,12 +5306,12 @@
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>DC - CLD (Quận 7)-(Trả Thùng xanh)</t>
+          <t>DC - LVT (Lê Văn Thọ)</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>-4567680972</t>
+          <t>-716998041</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H143" s="3" t="inlineStr"/>
@@ -5340,25 +5340,23 @@
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>DC - DS3 (Thủ đức)-(Trả Thùng Xanh)</t>
+          <t>DC - LVY (236A Lê Văn Sỹ)</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>-1001984727983</t>
+          <t>-5406820158</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="n">
-        <v>22</v>
-      </c>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr"/>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H144" s="3" t="inlineStr"/>
@@ -5374,25 +5372,25 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>DC - ECG (Eco Green)</t>
+          <t>DC - LVY (236A Lê Văn Sỹ)</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>-918508542</t>
+          <t>-1003958612570</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H145" s="3" t="inlineStr"/>
@@ -5408,12 +5406,12 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>DC - HMN (Harmona)</t>
+          <t>DC - NHG (Nguyên Hồng)</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>-4096943078</t>
+          <t>-787138197</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
@@ -5422,11 +5420,11 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H146" s="3" t="inlineStr"/>
@@ -5442,25 +5440,25 @@
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>DC - HTP (571 Huỳnh Tấn Phát)</t>
+          <t>DC - NKM(371 Nguyễn Kiệm)</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>-1001695487862</t>
+          <t>-733176842</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F147" s="2" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H147" s="3" t="inlineStr"/>
@@ -5476,12 +5474,12 @@
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>DC - KHI (98 Khánh Hội)</t>
+          <t>DC - NTD (160A Nguyễn Thị Định)</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>-4039116350</t>
+          <t>-641193549</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -5490,11 +5488,11 @@
         </is>
       </c>
       <c r="F148" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H148" s="3" t="inlineStr"/>
@@ -5510,25 +5508,25 @@
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>DC - LTC (97 Lê Thị Chợ)</t>
+          <t>DC - NTN (Nguyễn Trọng Tuyển)</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>-4115684818</t>
+          <t>-1004389700726</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H149" s="3" t="inlineStr"/>
@@ -5544,25 +5542,25 @@
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>DC - LTC (Lê Thị Chợ)</t>
+          <t>DC - NVT Q9 (367 Nguyễn Văn Tăng)</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>-1004451611911</t>
+          <t>-553882113</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H150" s="3" t="inlineStr"/>
@@ -5578,12 +5576,12 @@
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>DC - LVT (Lê Văn Thọ)</t>
+          <t>DC - PGS (Pegasuite)</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>-716998041</t>
+          <t>-4021539603</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
@@ -5592,11 +5590,11 @@
         </is>
       </c>
       <c r="F151" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H151" s="3" t="inlineStr"/>
@@ -5612,25 +5610,25 @@
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>DC - LVY (236A Lê Văn Sỹ)</t>
+          <t>DC - PHG (Bình chánh)-(Trả tote-rổ)</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>-1003958612570</t>
+          <t>-789904409</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H152" s="3" t="inlineStr"/>
@@ -5646,12 +5644,12 @@
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>DC - LVY (236A Lê Văn Sỹ)</t>
+          <t>DC - PHL (Phạm Hữu Lầu Q7)</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>-5406820158</t>
+          <t>-800905437</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -5659,10 +5657,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F153" s="2" t="inlineStr"/>
+      <c r="F153" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H153" s="3" t="inlineStr"/>
@@ -5678,17 +5678,17 @@
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>DC - NHG (Nguyên Hồng)</t>
+          <t>DC - Q50 (Quốc Lộ 50)</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>-787138197</t>
+          <t>-1004301337474</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F154" s="2" t="n">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H154" s="3" t="inlineStr"/>
@@ -5712,12 +5712,12 @@
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>DC - NKM(371 Nguyễn Kiệm)</t>
+          <t>DC - Q50 (Quốc Lộ 50)</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>-733176842</t>
+          <t>-5478025073</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -5725,12 +5725,10 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F155" s="2" t="n">
-        <v>24</v>
-      </c>
+      <c r="F155" s="2" t="inlineStr"/>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H155" s="3" t="inlineStr"/>
@@ -5746,12 +5744,12 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>DC - NTD (160A Nguyễn Thị Định)</t>
+          <t>DC - RS4 (Richstar)</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>-641193549</t>
+          <t>-4097859557</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -5760,11 +5758,11 @@
         </is>
       </c>
       <c r="F156" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H156" s="3" t="inlineStr"/>
@@ -5780,25 +5778,25 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>DC - NTN (Nguyễn Trọng Tuyển)</t>
+          <t>DC - SFR (D1 Safira)</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>-1004389700726</t>
+          <t>-4197902636</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F157" s="2" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H157" s="3" t="inlineStr"/>
@@ -5814,25 +5812,25 @@
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>DC - NVT Q9 (367 Nguyễn Văn Tăng)</t>
+          <t>DC - TMY(31 Tân Mỹ)</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>-553882113</t>
+          <t>-1001796134425</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H158" s="3" t="inlineStr"/>
@@ -5848,25 +5846,25 @@
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>DC - PGS (Pegasuite)</t>
+          <t>DC - TNT (195 Thống Nhất)</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>-4021539603</t>
+          <t>-1001844940870</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F159" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H159" s="3" t="inlineStr"/>
@@ -5882,12 +5880,12 @@
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>DC - PHG (Bình chánh)-(Trả tote-rổ)</t>
+          <t>DC - VH3 (S1.05 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>-789904409</t>
+          <t>-4056652819</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
@@ -5896,11 +5894,11 @@
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H160" s="3" t="inlineStr"/>
@@ -5916,12 +5914,12 @@
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>DC - PHL (Phạm Hữu Lầu Q7)</t>
+          <t>DC - VH5 (S03.05 Vinhomes)</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>-800905437</t>
+          <t>-5564355018</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
@@ -5929,12 +5927,10 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F161" s="2" t="n">
-        <v>17</v>
-      </c>
+      <c r="F161" s="2" t="inlineStr"/>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H161" s="3" t="inlineStr"/>
@@ -5950,12 +5946,12 @@
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>DC - Q50 (Quốc Lộ 50)</t>
+          <t>DC - VH5 (S03.05 Vinhomes)</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>-1004301337474</t>
+          <t>-1004357370577</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
@@ -5964,11 +5960,11 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H162" s="3" t="inlineStr"/>
@@ -5984,12 +5980,12 @@
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>DC - Q50 (Quốc Lộ 50)</t>
+          <t>DC - VHT(54 Vũ Huy Tấn)</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>-5478025073</t>
+          <t>-636891030</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
@@ -5997,10 +5993,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr"/>
+      <c r="F163" s="2" t="n">
+        <v>28</v>
+      </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H163" s="3" t="inlineStr"/>
@@ -6016,12 +6014,12 @@
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>DC - RS4 (Richstar)</t>
+          <t>DC - VLA (128 Vườn Lài)</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>-4097859557</t>
+          <t>-4186843633</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
@@ -6034,7 +6032,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H164" s="3" t="inlineStr"/>
@@ -6050,12 +6048,12 @@
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>DC - SFR (D1 Safira)</t>
+          <t>DC-ACU- 01 Chung cư An Cư An Phú</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>-4197902636</t>
+          <t>-4578848570</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
@@ -6064,11 +6062,11 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H165" s="3" t="inlineStr"/>
@@ -6084,25 +6082,25 @@
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>DC - STORE - SOE</t>
+          <t>DC-BTH</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>-1001632996518</t>
+          <t>-4854369578</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>493</v>
+        <v>19</v>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H166" s="3" t="inlineStr"/>
@@ -6118,12 +6116,12 @@
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>DC - TMY(31 Tân Mỹ)</t>
+          <t>DC-EMR (BD) (Trả tote-rổ)</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>-1001796134425</t>
+          <t>-1002686145863</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
@@ -6132,11 +6130,11 @@
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H167" s="3" t="inlineStr"/>
@@ -6152,25 +6150,25 @@
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>DC - TNT (195 Thống Nhất)</t>
+          <t>DC-HTC</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>-1001844940870</t>
+          <t>-4832751364</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H168" s="3" t="inlineStr"/>
@@ -6186,12 +6184,12 @@
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>DC - VH3 (S1.05 Vinhomes Grand Park)</t>
+          <t>DC-HV2</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>-4056652819</t>
+          <t>-4836039448</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
@@ -6200,11 +6198,11 @@
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr"/>
@@ -6220,25 +6218,25 @@
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>DC - VH5 (S03.05 Vinhomes)</t>
+          <t>DC-NVK</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>-1004357370577</t>
+          <t>-4827088164</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H170" s="3" t="inlineStr"/>
@@ -6254,12 +6252,12 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>DC - VH5 (S03.05 Vinhomes)</t>
+          <t>DC-PPZ</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>-5564355018</t>
+          <t>-4972623393</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
@@ -6267,10 +6265,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F171" s="2" t="inlineStr"/>
+      <c r="F171" s="2" t="n">
+        <v>20</v>
+      </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H171" s="3" t="inlineStr"/>
@@ -6286,12 +6286,12 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>DC - VHT(54 Vũ Huy Tấn)</t>
+          <t>DC-PVB</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>-636891030</t>
+          <t>-4724011528</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H172" s="3" t="inlineStr"/>
@@ -6320,12 +6320,12 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>DC - VLA (128 Vườn Lài)</t>
+          <t>DC-SCV</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>-4186843633</t>
+          <t>-4922136877</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
@@ -6334,11 +6334,11 @@
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H173" s="3" t="inlineStr"/>
@@ -6354,25 +6354,25 @@
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>DC FRESH - KẾ TOÁN</t>
+          <t>DC-THN</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>-1003601660322</t>
+          <t>-4982081891</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H174" s="3" t="inlineStr"/>
@@ -6388,12 +6388,12 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>DC FRESH - KẾ TOÁN</t>
+          <t>DMR - DC (Block C Diamond Riverside)</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>-595120296</t>
+          <t>-4883865942</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -6401,10 +6401,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr"/>
+      <c r="F175" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H175" s="3" t="inlineStr"/>
@@ -6420,25 +6422,25 @@
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>DC x KFM - Cân tồn tháng - Phiếu hủy</t>
+          <t>DS7 - DC (99 Đường Số 7)</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>-5006191213</t>
+          <t>-1002166724266</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H176" s="3" t="inlineStr"/>
@@ -6454,12 +6456,12 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>DC x SCM Kiểm tra XNT phiếu pending</t>
+          <t>EH3- DC</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>-5201470520</t>
+          <t>-4712243485</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -6468,11 +6470,11 @@
         </is>
       </c>
       <c r="F177" s="2" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H177" s="3" t="inlineStr"/>
@@ -6488,12 +6490,12 @@
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>DC-ACU- 01 Chung cư An Cư An Phú</t>
+          <t>GHA - DC (The Art Gia Hòa)</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>-4578848570</t>
+          <t>-4125880558</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -6502,11 +6504,11 @@
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H178" s="3" t="inlineStr"/>
@@ -6522,25 +6524,25 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>DC-BTH</t>
+          <t>HHM - DC (165 Hoàng Hoa Thám)</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>-4854369578</t>
+          <t>-1003822384320</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H179" s="3" t="inlineStr"/>
@@ -6556,25 +6558,23 @@
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>DC-EMR (BD) (Trả tote-rổ)</t>
+          <t>HHM - DC (165 Hoàng Hoa Thám)</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>-1002686145863</t>
+          <t>-4612672037</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="n">
-        <v>19</v>
-      </c>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr"/>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H180" s="3" t="inlineStr"/>
@@ -6590,12 +6590,12 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>DC-HTC</t>
+          <t>HLR - DC ( Block A Himlam Riverside Q7)</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>-4832751364</t>
+          <t>-4943081238</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
@@ -6604,11 +6604,11 @@
         </is>
       </c>
       <c r="F181" s="2" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H181" s="3" t="inlineStr"/>
@@ -6624,12 +6624,12 @@
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>DC-HV2</t>
+          <t>HPD - DC (01-06 TMDV Him Lam Phú Đông)</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>-4836039448</t>
+          <t>-4820723298</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -6638,11 +6638,11 @@
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H182" s="3" t="inlineStr"/>
@@ -6658,12 +6658,12 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>DC-NVK</t>
+          <t>HTN - DC (17 Hồ Thị Nhung)</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>-4827088164</t>
+          <t>-4658447671</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
@@ -6672,11 +6672,11 @@
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H183" s="3" t="inlineStr"/>
@@ -6692,12 +6692,12 @@
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>DC-PPZ</t>
+          <t>KDG - DC (10D Kỳ Đồng)</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>-4972623393</t>
+          <t>-4951125300</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -6706,11 +6706,11 @@
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H184" s="3" t="inlineStr"/>
@@ -6726,12 +6726,12 @@
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>DC-PVB</t>
+          <t>LVH - DC (222 Lê Văn Thịnh)</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>-4724011528</t>
+          <t>-4614044179</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -6740,11 +6740,11 @@
         </is>
       </c>
       <c r="F185" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H185" s="3" t="inlineStr"/>
@@ -6760,12 +6760,12 @@
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>DC-SCV</t>
+          <t>LVL - DC (166E Lê Văn Lương)</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>-4922136877</t>
+          <t>-884744948</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
@@ -6774,11 +6774,11 @@
         </is>
       </c>
       <c r="F186" s="2" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H186" s="3" t="inlineStr"/>
@@ -6794,12 +6794,12 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>DC-THN</t>
+          <t>MZ2 - DC (A7-8 Valora Mizuki)</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>-4982081891</t>
+          <t>-4906931555</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
@@ -6808,11 +6808,11 @@
         </is>
       </c>
       <c r="F187" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H187" s="3" t="inlineStr"/>
@@ -6828,12 +6828,12 @@
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>DMR - DC (Block C Diamond Riverside)</t>
+          <t>MZK - DC (TMDV2 Mizuki Park)</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>-4883865942</t>
+          <t>-4097174073</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
@@ -6842,11 +6842,11 @@
         </is>
       </c>
       <c r="F188" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H188" s="3" t="inlineStr"/>
@@ -6862,25 +6862,25 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>DS7 - DC (99 Đường Số 7)</t>
+          <t>NDH - DC (1426 Nguyễn Duy Trinh)</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>-1002166724266</t>
+          <t>-4641160091</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F189" s="2" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H189" s="3" t="inlineStr"/>
@@ -6896,12 +6896,12 @@
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Dán tem + lên tồn hệ thống_Kho CCDC</t>
+          <t>NTO - DC (108 Ngô Tất Tố)</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>-4950281745</t>
+          <t>-4870440616</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
@@ -6910,11 +6910,11 @@
         </is>
       </c>
       <c r="F190" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H190" s="3" t="inlineStr"/>
@@ -6930,25 +6930,25 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>EH3- DC</t>
+          <t>NTU - DC (46 Nguyễn Thị Tú)</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>-4712243485</t>
+          <t>-1001929557412</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F191" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H191" s="3" t="inlineStr"/>
@@ -6964,12 +6964,12 @@
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>GHA - DC (The Art Gia Hòa)</t>
+          <t>NVD - DC (42 Nguyễn Văn Đậu)</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>-4125880558</t>
+          <t>-4246704011</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
@@ -6978,11 +6978,11 @@
         </is>
       </c>
       <c r="F192" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H192" s="3" t="inlineStr"/>
@@ -6998,25 +6998,25 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>HHM - DC (165 Hoàng Hoa Thám)</t>
+          <t>Q7R - DC (Lô CD L1-12 Q7 Riverside Đào Trí)</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>-1003822384320</t>
+          <t>-4610245241</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F193" s="2" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H193" s="3" t="inlineStr"/>
@@ -7032,12 +7032,12 @@
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>HHM - DC (165 Hoàng Hoa Thám)</t>
+          <t>QHG_DC_ store</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>-4612672037</t>
+          <t>-4249658669</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
@@ -7045,10 +7045,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr"/>
+      <c r="F194" s="2" t="n">
+        <v>24</v>
+      </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H194" s="3" t="inlineStr"/>
@@ -7064,12 +7066,12 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>HLR - DC ( Block A Himlam Riverside Q7)</t>
+          <t>RVS - DC (C0.01 Riverside Phú Mỹ Hưng)</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>-4943081238</t>
+          <t>-4928360925</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -7078,11 +7080,11 @@
         </is>
       </c>
       <c r="F195" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H195" s="3" t="inlineStr"/>
@@ -7098,12 +7100,12 @@
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>HPD - DC (01-06 TMDV Him Lam Phú Đông)</t>
+          <t>VH2 - DC (S10.02 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>-4820723298</t>
+          <t>-4077409269</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -7112,11 +7114,11 @@
         </is>
       </c>
       <c r="F196" s="2" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H196" s="3" t="inlineStr"/>
@@ -7132,12 +7134,12 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>HTN - DC (17 Hồ Thị Nhung)</t>
+          <t>VH5 - DC (S03.05 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>-4658447671</t>
+          <t>-4971875234</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
@@ -7146,11 +7148,11 @@
         </is>
       </c>
       <c r="F197" s="2" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H197" s="3" t="inlineStr"/>
@@ -7166,12 +7168,12 @@
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Hậu kiểm kho rau</t>
+          <t>VH7 - DC (BS11 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>-5044734031</t>
+          <t>-4873359487</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -7180,11 +7182,11 @@
         </is>
       </c>
       <c r="F198" s="2" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H198" s="3" t="inlineStr"/>
@@ -7200,12 +7202,12 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>KDG - DC (10D Kỳ Đồng)</t>
+          <t>VPC - DC (02 Nguyễn Thị Nhung)</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>-4951125300</t>
+          <t>-4587582513</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
@@ -7213,12 +7215,10 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F199" s="2" t="n">
-        <v>17</v>
-      </c>
+      <c r="F199" s="2" t="inlineStr"/>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>DC (200)</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H199" s="3" t="inlineStr"/>
@@ -7234,12 +7234,12 @@
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>KFM - SCF: CHUYỂN HÀNG DC KHÔ</t>
+          <t>VPC - DC (02 Nguyễn Thị Nhung)</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>-1001726689633</t>
+          <t>-1003925120550</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
@@ -7248,896 +7248,14 @@
         </is>
       </c>
       <c r="F200" s="2" t="n">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>Khác / Overflow</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H200" s="3" t="inlineStr"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="B201" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>KFM x AIDI x DC - OPS</t>
-        </is>
-      </c>
-      <c r="D201" s="2" t="inlineStr">
-        <is>
-          <t>-4645689451</t>
-        </is>
-      </c>
-      <c r="E201" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F201" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="G201" s="2" t="inlineStr">
-        <is>
-          <t>Khác / Overflow</t>
-        </is>
-      </c>
-      <c r="H201" s="3" t="inlineStr"/>
-    </row>
-    <row r="202">
-      <c r="A202" s="2" t="n">
-        <v>201</v>
-      </c>
-      <c r="B202" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C202" s="3" t="inlineStr">
-        <is>
-          <t>KSCxx.xx Quản Lý Tồn Kho</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr">
-        <is>
-          <t>-1004478237467</t>
-        </is>
-      </c>
-      <c r="E202" s="2" t="inlineStr">
-        <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F202" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="G202" s="2" t="inlineStr">
-        <is>
-          <t>Khác / Overflow</t>
-        </is>
-      </c>
-      <c r="H202" s="3" t="inlineStr"/>
-    </row>
-    <row r="203">
-      <c r="A203" s="2" t="n">
-        <v>202</v>
-      </c>
-      <c r="B203" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C203" s="3" t="inlineStr">
-        <is>
-          <t>LVH - DC (222 Lê Văn Thịnh)</t>
-        </is>
-      </c>
-      <c r="D203" s="2" t="inlineStr">
-        <is>
-          <t>-4614044179</t>
-        </is>
-      </c>
-      <c r="E203" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F203" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="G203" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H203" s="3" t="inlineStr"/>
-    </row>
-    <row r="204">
-      <c r="A204" s="2" t="n">
-        <v>203</v>
-      </c>
-      <c r="B204" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C204" s="3" t="inlineStr">
-        <is>
-          <t>LVL - DC (166E Lê Văn Lương)</t>
-        </is>
-      </c>
-      <c r="D204" s="2" t="inlineStr">
-        <is>
-          <t>-884744948</t>
-        </is>
-      </c>
-      <c r="E204" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F204" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="G204" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H204" s="3" t="inlineStr"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="2" t="n">
-        <v>204</v>
-      </c>
-      <c r="B205" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C205" s="3" t="inlineStr">
-        <is>
-          <t>Logistic KFM</t>
-        </is>
-      </c>
-      <c r="D205" s="2" t="inlineStr">
-        <is>
-          <t>-4795315212</t>
-        </is>
-      </c>
-      <c r="E205" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F205" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="G205" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H205" s="3" t="inlineStr"/>
-    </row>
-    <row r="206">
-      <c r="A206" s="2" t="n">
-        <v>205</v>
-      </c>
-      <c r="B206" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C206" s="3" t="inlineStr">
-        <is>
-          <t>Logistic _ inventory</t>
-        </is>
-      </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>-1003951952395</t>
-        </is>
-      </c>
-      <c r="E206" s="2" t="inlineStr">
-        <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F206" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="G206" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H206" s="3" t="inlineStr"/>
-    </row>
-    <row r="207">
-      <c r="A207" s="2" t="n">
-        <v>206</v>
-      </c>
-      <c r="B207" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C207" s="3" t="inlineStr">
-        <is>
-          <t>Logistics Team_Intern</t>
-        </is>
-      </c>
-      <c r="D207" s="2" t="inlineStr">
-        <is>
-          <t>-5580654562</t>
-        </is>
-      </c>
-      <c r="E207" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F207" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G207" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H207" s="3" t="inlineStr"/>
-    </row>
-    <row r="208">
-      <c r="A208" s="2" t="n">
-        <v>207</v>
-      </c>
-      <c r="B208" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C208" s="3" t="inlineStr">
-        <is>
-          <t>MZ2 - DC (A7-8 Valora Mizuki)</t>
-        </is>
-      </c>
-      <c r="D208" s="2" t="inlineStr">
-        <is>
-          <t>-4906931555</t>
-        </is>
-      </c>
-      <c r="E208" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F208" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G208" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H208" s="3" t="inlineStr"/>
-    </row>
-    <row r="209">
-      <c r="A209" s="2" t="n">
-        <v>208</v>
-      </c>
-      <c r="B209" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C209" s="3" t="inlineStr">
-        <is>
-          <t>MZK - DC (TMDV2 Mizuki Park)</t>
-        </is>
-      </c>
-      <c r="D209" s="2" t="inlineStr">
-        <is>
-          <t>-4097174073</t>
-        </is>
-      </c>
-      <c r="E209" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F209" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G209" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H209" s="3" t="inlineStr"/>
-    </row>
-    <row r="210">
-      <c r="A210" s="2" t="n">
-        <v>209</v>
-      </c>
-      <c r="B210" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C210" s="3" t="inlineStr">
-        <is>
-          <t>NDH - DC (1426 Nguyễn Duy Trinh)</t>
-        </is>
-      </c>
-      <c r="D210" s="2" t="inlineStr">
-        <is>
-          <t>-4641160091</t>
-        </is>
-      </c>
-      <c r="E210" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F210" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="G210" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H210" s="3" t="inlineStr"/>
-    </row>
-    <row r="211">
-      <c r="A211" s="2" t="n">
-        <v>210</v>
-      </c>
-      <c r="B211" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C211" s="3" t="inlineStr">
-        <is>
-          <t>NSO- KFM- BDU- TAN - 275 D33 KDC Viet Sing Khai Trương 9/10/2026</t>
-        </is>
-      </c>
-      <c r="D211" s="2" t="inlineStr">
-        <is>
-          <t>-1003793951751</t>
-        </is>
-      </c>
-      <c r="E211" s="2" t="inlineStr">
-        <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F211" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="G211" s="2" t="inlineStr">
-        <is>
-          <t>Khác / Overflow</t>
-        </is>
-      </c>
-      <c r="H211" s="3" t="inlineStr"/>
-    </row>
-    <row r="212">
-      <c r="A212" s="2" t="n">
-        <v>211</v>
-      </c>
-      <c r="B212" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C212" s="3" t="inlineStr">
-        <is>
-          <t>NTO - DC (108 Ngô Tất Tố)</t>
-        </is>
-      </c>
-      <c r="D212" s="2" t="inlineStr">
-        <is>
-          <t>-4870440616</t>
-        </is>
-      </c>
-      <c r="E212" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F212" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="G212" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H212" s="3" t="inlineStr"/>
-    </row>
-    <row r="213">
-      <c r="A213" s="2" t="n">
-        <v>212</v>
-      </c>
-      <c r="B213" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C213" s="3" t="inlineStr">
-        <is>
-          <t>NTU - DC (46 Nguyễn Thị Tú)</t>
-        </is>
-      </c>
-      <c r="D213" s="2" t="inlineStr">
-        <is>
-          <t>-1001929557412</t>
-        </is>
-      </c>
-      <c r="E213" s="2" t="inlineStr">
-        <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F213" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G213" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H213" s="3" t="inlineStr"/>
-    </row>
-    <row r="214">
-      <c r="A214" s="2" t="n">
-        <v>213</v>
-      </c>
-      <c r="B214" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C214" s="3" t="inlineStr">
-        <is>
-          <t>NVD - DC (42 Nguyễn Văn Đậu)</t>
-        </is>
-      </c>
-      <c r="D214" s="2" t="inlineStr">
-        <is>
-          <t>-4246704011</t>
-        </is>
-      </c>
-      <c r="E214" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F214" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G214" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H214" s="3" t="inlineStr"/>
-    </row>
-    <row r="215">
-      <c r="A215" s="2" t="n">
-        <v>214</v>
-      </c>
-      <c r="B215" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C215" s="3" t="inlineStr">
-        <is>
-          <t>Nhập - Chuyển - Xuất CCDC (3H)</t>
-        </is>
-      </c>
-      <c r="D215" s="2" t="inlineStr">
-        <is>
-          <t>-4234575718</t>
-        </is>
-      </c>
-      <c r="E215" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F215" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G215" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H215" s="3" t="inlineStr"/>
-    </row>
-    <row r="216">
-      <c r="A216" s="2" t="n">
-        <v>215</v>
-      </c>
-      <c r="B216" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C216" s="3" t="inlineStr">
-        <is>
-          <t>Q7R - DC (Lô CD L1-12 Q7 Riverside Đào Trí)</t>
-        </is>
-      </c>
-      <c r="D216" s="2" t="inlineStr">
-        <is>
-          <t>-4610245241</t>
-        </is>
-      </c>
-      <c r="E216" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F216" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G216" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H216" s="3" t="inlineStr"/>
-    </row>
-    <row r="217">
-      <c r="A217" s="2" t="n">
-        <v>216</v>
-      </c>
-      <c r="B217" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C217" s="3" t="inlineStr">
-        <is>
-          <t>QHG_DC_ store</t>
-        </is>
-      </c>
-      <c r="D217" s="2" t="inlineStr">
-        <is>
-          <t>-4249658669</t>
-        </is>
-      </c>
-      <c r="E217" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F217" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="G217" s="2" t="inlineStr">
-        <is>
-          <t>Khác / Overflow</t>
-        </is>
-      </c>
-      <c r="H217" s="3" t="inlineStr"/>
-    </row>
-    <row r="218">
-      <c r="A218" s="2" t="n">
-        <v>217</v>
-      </c>
-      <c r="B218" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C218" s="3" t="inlineStr">
-        <is>
-          <t>RVS - DC (C0.01 Riverside Phú Mỹ Hưng)</t>
-        </is>
-      </c>
-      <c r="D218" s="2" t="inlineStr">
-        <is>
-          <t>-4928360925</t>
-        </is>
-      </c>
-      <c r="E218" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F218" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="G218" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H218" s="3" t="inlineStr"/>
-    </row>
-    <row r="219">
-      <c r="A219" s="2" t="n">
-        <v>218</v>
-      </c>
-      <c r="B219" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C219" s="3" t="inlineStr">
-        <is>
-          <t>Report logistic</t>
-        </is>
-      </c>
-      <c r="D219" s="2" t="inlineStr">
-        <is>
-          <t>-5221667525</t>
-        </is>
-      </c>
-      <c r="E219" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F219" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="G219" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H219" s="3" t="inlineStr"/>
-    </row>
-    <row r="220">
-      <c r="A220" s="2" t="n">
-        <v>219</v>
-      </c>
-      <c r="B220" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C220" s="3" t="inlineStr">
-        <is>
-          <t>SCF x KFM - Kho Đông Hưng - SETUP SWAT</t>
-        </is>
-      </c>
-      <c r="D220" s="2" t="inlineStr">
-        <is>
-          <t>-5223681988</t>
-        </is>
-      </c>
-      <c r="E220" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F220" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="G220" s="2" t="inlineStr">
-        <is>
-          <t>Khác / Overflow</t>
-        </is>
-      </c>
-      <c r="H220" s="3" t="inlineStr"/>
-    </row>
-    <row r="221">
-      <c r="A221" s="2" t="n">
-        <v>220</v>
-      </c>
-      <c r="B221" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C221" s="3" t="inlineStr">
-        <is>
-          <t>Support Kho ITL - KFM</t>
-        </is>
-      </c>
-      <c r="D221" s="2" t="inlineStr">
-        <is>
-          <t>-4649086309</t>
-        </is>
-      </c>
-      <c r="E221" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F221" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="G221" s="2" t="inlineStr">
-        <is>
-          <t>Khác / Overflow</t>
-        </is>
-      </c>
-      <c r="H221" s="3" t="inlineStr"/>
-    </row>
-    <row r="222">
-      <c r="A222" s="2" t="n">
-        <v>221</v>
-      </c>
-      <c r="B222" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C222" s="3" t="inlineStr">
-        <is>
-          <t>VH2 - DC (S10.02 Vinhomes Grand Park)</t>
-        </is>
-      </c>
-      <c r="D222" s="2" t="inlineStr">
-        <is>
-          <t>-4077409269</t>
-        </is>
-      </c>
-      <c r="E222" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F222" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G222" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H222" s="3" t="inlineStr"/>
-    </row>
-    <row r="223">
-      <c r="A223" s="2" t="n">
-        <v>222</v>
-      </c>
-      <c r="B223" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C223" s="3" t="inlineStr">
-        <is>
-          <t>VH5 - DC (S03.05 Vinhomes Grand Park)</t>
-        </is>
-      </c>
-      <c r="D223" s="2" t="inlineStr">
-        <is>
-          <t>-4971875234</t>
-        </is>
-      </c>
-      <c r="E223" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F223" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="G223" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H223" s="3" t="inlineStr"/>
-    </row>
-    <row r="224">
-      <c r="A224" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="B224" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C224" s="3" t="inlineStr">
-        <is>
-          <t>VH7 - DC (BS11 Vinhomes Grand Park)</t>
-        </is>
-      </c>
-      <c r="D224" s="2" t="inlineStr">
-        <is>
-          <t>-4873359487</t>
-        </is>
-      </c>
-      <c r="E224" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F224" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G224" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H224" s="3" t="inlineStr"/>
-    </row>
-    <row r="225">
-      <c r="A225" s="2" t="n">
-        <v>224</v>
-      </c>
-      <c r="B225" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C225" s="3" t="inlineStr">
-        <is>
-          <t>VPC - DC (02 Nguyễn Thị Nhung)</t>
-        </is>
-      </c>
-      <c r="D225" s="2" t="inlineStr">
-        <is>
-          <t>-1003925120550</t>
-        </is>
-      </c>
-      <c r="E225" s="2" t="inlineStr">
-        <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F225" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G225" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H225" s="3" t="inlineStr"/>
-    </row>
-    <row r="226">
-      <c r="A226" s="2" t="n">
-        <v>225</v>
-      </c>
-      <c r="B226" s="2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C226" s="3" t="inlineStr">
-        <is>
-          <t>VPC - DC (02 Nguyễn Thị Nhung)</t>
-        </is>
-      </c>
-      <c r="D226" s="2" t="inlineStr">
-        <is>
-          <t>-4587582513</t>
-        </is>
-      </c>
-      <c r="E226" s="2" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F226" s="2" t="inlineStr"/>
-      <c r="G226" s="2" t="inlineStr">
-        <is>
-          <t>DC (200)</t>
-        </is>
-      </c>
-      <c r="H226" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Them nhom DC - HMN (Harmona) vao folder DC va cap nhat file Excel len 200 nhom
</commit_message>
<xml_diff>
--- a/Danh_Sach_Chat_ID_Nhom_DC.xlsx
+++ b/Danh_Sach_Chat_ID_Nhom_DC.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DANH_SACH_DC_199" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DANH_SACH_DC_200" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4689,17 +4689,17 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>HMN</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>AV4 - DC (SAV_04-00.03 The Sun Avenue)</t>
+          <t>DC - HMN (Harmona)</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>-4903740099</t>
+          <t>-4096943078</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H125" s="3" t="inlineStr"/>
@@ -4728,12 +4728,12 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>CHR - DC (S01.11 Block A1 Charm Sapphire)</t>
+          <t>AV4 - DC (SAV_04-00.03 The Sun Avenue)</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>-4946147649</t>
+          <t>-4903740099</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
@@ -4762,12 +4762,12 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>CKO - DC (85 Cây Keo)</t>
+          <t>CHR - DC (S01.11 Block A1 Charm Sapphire)</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>-613928063</t>
+          <t>-4946147649</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="F127" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
@@ -4796,12 +4796,12 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>CLG - DC (64A Cửu Long)</t>
+          <t>CKO - DC (85 Cây Keo)</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>-4864768952</t>
+          <t>-613928063</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -4810,7 +4810,7 @@
         </is>
       </c>
       <c r="F128" s="2" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
@@ -4830,12 +4830,12 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>CLN - DC</t>
+          <t>CLG - DC (64A Cửu Long)</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>-4870092396</t>
+          <t>-4864768952</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -4844,11 +4844,11 @@
         </is>
       </c>
       <c r="F129" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H129" s="3" t="inlineStr"/>
@@ -4864,12 +4864,12 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>CN1 - DC (48 CN1)</t>
+          <t>CLN - DC</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>-868672635</t>
+          <t>-4870092396</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -4878,11 +4878,11 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H130" s="3" t="inlineStr"/>
@@ -4898,12 +4898,12 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>CTH - DC (TMDV Citihome Cát Lái)</t>
+          <t>CN1 - DC (48 CN1)</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>-4117975293</t>
+          <t>-868672635</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="F131" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
@@ -4932,12 +4932,12 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>D10 - DC (01 Đường Số 10 Tân Kiểng)</t>
+          <t>CTH - DC (TMDV Citihome Cát Lái)</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>-4950196076</t>
+          <t>-4117975293</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -4946,7 +4946,7 @@
         </is>
       </c>
       <c r="F132" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
@@ -4966,25 +4966,25 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>DC - 410 PHI (410 Phan Huy Ích)</t>
+          <t>D10 - DC (01 Đường Số 10 Tân Kiểng)</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>-1001878454662</t>
+          <t>-4950196076</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H133" s="3" t="inlineStr"/>
@@ -5000,21 +5000,21 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>DC - AKR (Akari City)</t>
+          <t>DC - 410 PHI (410 Phan Huy Ích)</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>-4114032701</t>
+          <t>-1001878454662</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
@@ -5034,21 +5034,21 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>DC - BQI (Quận BT) - (Trả tote và rổ)</t>
+          <t>DC - AKR (Akari City)</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>-1001838756395</t>
+          <t>-4114032701</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F135" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
@@ -5068,25 +5068,25 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>DC - CLD (Quận 7)-(Trả Thùng xanh)</t>
+          <t>DC - BQI (Quận BT) - (Trả tote và rổ)</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>-4567680972</t>
+          <t>-1001838756395</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H136" s="3" t="inlineStr"/>
@@ -5102,21 +5102,21 @@
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>DC - DS3 (Thủ đức)-(Trả Thùng Xanh)</t>
+          <t>DC - CLD (Quận 7)-(Trả Thùng xanh)</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>-1001984727983</t>
+          <t>-4567680972</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F137" s="2" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
@@ -5136,21 +5136,21 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>DC - ECG (Eco Green)</t>
+          <t>DC - DS3 (Thủ đức)-(Trả Thùng Xanh)</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>-918508542</t>
+          <t>-1001984727983</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
@@ -5170,17 +5170,17 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>DC - HTP (571 Huỳnh Tấn Phát)</t>
+          <t>DC - ECG (Eco Green)</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>-1001695487862</t>
+          <t>-918508542</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F139" s="2" t="n">
@@ -5204,25 +5204,25 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>DC - KHI (98 Khánh Hội)</t>
+          <t>DC - HTP (571 Huỳnh Tấn Phát)</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>-4039116350</t>
+          <t>-1001695487862</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H140" s="3" t="inlineStr"/>
@@ -5238,12 +5238,12 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>DC - LTC (97 Lê Thị Chợ)</t>
+          <t>DC - KHI (98 Khánh Hội)</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>-4115684818</t>
+          <t>-4039116350</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
@@ -5252,11 +5252,11 @@
         </is>
       </c>
       <c r="F141" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H141" s="3" t="inlineStr"/>
@@ -5272,21 +5272,21 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>DC - LTC (Lê Thị Chợ)</t>
+          <t>DC - LTC (97 Lê Thị Chợ)</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>-1004451611911</t>
+          <t>-4115684818</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
@@ -5306,25 +5306,25 @@
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>DC - LVT (Lê Văn Thọ)</t>
+          <t>DC - LTC (Lê Thị Chợ)</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>-716998041</t>
+          <t>-1004451611911</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H143" s="3" t="inlineStr"/>
@@ -5340,12 +5340,12 @@
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>DC - LVY (236A Lê Văn Sỹ)</t>
+          <t>DC - LVT (Lê Văn Thọ)</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>-5406820158</t>
+          <t>-716998041</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -5353,10 +5353,12 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="n">
+        <v>24</v>
+      </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H144" s="3" t="inlineStr"/>
@@ -5377,17 +5379,15 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>-1003958612570</t>
+          <t>-5406820158</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F145" s="2" t="n">
-        <v>32</v>
-      </c>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr"/>
       <c r="G145" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -5406,21 +5406,21 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>DC - NHG (Nguyên Hồng)</t>
+          <t>DC - LVY (236A Lê Văn Sỹ)</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>-787138197</t>
+          <t>-1003958612570</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
@@ -5440,12 +5440,12 @@
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>DC - NKM(371 Nguyễn Kiệm)</t>
+          <t>DC - NHG (Nguyên Hồng)</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>-733176842</t>
+          <t>-787138197</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
@@ -5454,7 +5454,7 @@
         </is>
       </c>
       <c r="F147" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
@@ -5474,12 +5474,12 @@
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>DC - NTD (160A Nguyễn Thị Định)</t>
+          <t>DC - NKM(371 Nguyễn Kiệm)</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>-641193549</t>
+          <t>-733176842</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -5488,7 +5488,7 @@
         </is>
       </c>
       <c r="F148" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
@@ -5508,21 +5508,21 @@
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>DC - NTN (Nguyễn Trọng Tuyển)</t>
+          <t>DC - NTD (160A Nguyễn Thị Định)</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>-1004389700726</t>
+          <t>-641193549</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
@@ -5542,21 +5542,21 @@
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>DC - NVT Q9 (367 Nguyễn Văn Tăng)</t>
+          <t>DC - NTN (Nguyễn Trọng Tuyển)</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>-553882113</t>
+          <t>-1004389700726</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
@@ -5576,12 +5576,12 @@
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>DC - PGS (Pegasuite)</t>
+          <t>DC - NVT Q9 (367 Nguyễn Văn Tăng)</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>-4021539603</t>
+          <t>-553882113</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="F151" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
@@ -5610,12 +5610,12 @@
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>DC - PHG (Bình chánh)-(Trả tote-rổ)</t>
+          <t>DC - PGS (Pegasuite)</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>-789904409</t>
+          <t>-4021539603</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -5624,11 +5624,11 @@
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H152" s="3" t="inlineStr"/>
@@ -5644,12 +5644,12 @@
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>DC - PHL (Phạm Hữu Lầu Q7)</t>
+          <t>DC - PHG (Bình chánh)-(Trả tote-rổ)</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>-800905437</t>
+          <t>-789904409</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -5658,11 +5658,11 @@
         </is>
       </c>
       <c r="F153" s="2" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H153" s="3" t="inlineStr"/>
@@ -5678,21 +5678,21 @@
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>DC - Q50 (Quốc Lộ 50)</t>
+          <t>DC - PHL (Phạm Hữu Lầu Q7)</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>-1004301337474</t>
+          <t>-800905437</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
@@ -5717,15 +5717,17 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>-5478025073</t>
+          <t>-1004301337474</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F155" s="2" t="inlineStr"/>
+          <t>Supergroup</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="n">
+        <v>23</v>
+      </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -5744,12 +5746,12 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>DC - RS4 (Richstar)</t>
+          <t>DC - Q50 (Quốc Lộ 50)</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>-4097859557</t>
+          <t>-5478025073</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -5757,9 +5759,7 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F156" s="2" t="n">
-        <v>21</v>
-      </c>
+      <c r="F156" s="2" t="inlineStr"/>
       <c r="G156" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -5778,12 +5778,12 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>DC - SFR (D1 Safira)</t>
+          <t>DC - RS4 (Richstar)</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>-4197902636</t>
+          <t>-4097859557</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
@@ -5792,7 +5792,7 @@
         </is>
       </c>
       <c r="F157" s="2" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
@@ -5812,21 +5812,21 @@
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>DC - TMY(31 Tân Mỹ)</t>
+          <t>DC - SFR (D1 Safira)</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>-1001796134425</t>
+          <t>-4197902636</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
@@ -5846,12 +5846,12 @@
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>DC - TNT (195 Thống Nhất)</t>
+          <t>DC - TMY(31 Tân Mỹ)</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>-1001844940870</t>
+          <t>-1001796134425</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -5860,7 +5860,7 @@
         </is>
       </c>
       <c r="F159" s="2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
@@ -5880,21 +5880,21 @@
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>DC - VH3 (S1.05 Vinhomes Grand Park)</t>
+          <t>DC - TNT (195 Thống Nhất)</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>-4056652819</t>
+          <t>-1001844940870</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
@@ -5914,12 +5914,12 @@
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>DC - VH5 (S03.05 Vinhomes)</t>
+          <t>DC - VH3 (S1.05 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>-5564355018</t>
+          <t>-4056652819</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
@@ -5927,7 +5927,9 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F161" s="2" t="inlineStr"/>
+      <c r="F161" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -5951,17 +5953,15 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>-1004357370577</t>
+          <t>-5564355018</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="n">
-        <v>27</v>
-      </c>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr"/>
       <c r="G162" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -5980,21 +5980,21 @@
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>DC - VHT(54 Vũ Huy Tấn)</t>
+          <t>DC - VH5 (S03.05 Vinhomes)</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>-636891030</t>
+          <t>-1004357370577</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
@@ -6014,12 +6014,12 @@
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>DC - VLA (128 Vườn Lài)</t>
+          <t>DC - VHT(54 Vũ Huy Tấn)</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>-4186843633</t>
+          <t>-636891030</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
@@ -6048,12 +6048,12 @@
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>DC-ACU- 01 Chung cư An Cư An Phú</t>
+          <t>DC - VLA (128 Vườn Lài)</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>-4578848570</t>
+          <t>-4186843633</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
@@ -6082,12 +6082,12 @@
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>DC-BTH</t>
+          <t>DC-ACU- 01 Chung cư An Cư An Phú</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>-4854369578</t>
+          <t>-4578848570</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
@@ -6096,7 +6096,7 @@
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
@@ -6116,17 +6116,17 @@
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>DC-EMR (BD) (Trả tote-rổ)</t>
+          <t>DC-BTH</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>-1002686145863</t>
+          <t>-4854369578</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F167" s="2" t="n">
@@ -6150,25 +6150,25 @@
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>DC-HTC</t>
+          <t>DC-EMR (BD) (Trả tote-rổ)</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>-4832751364</t>
+          <t>-1002686145863</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H168" s="3" t="inlineStr"/>
@@ -6184,12 +6184,12 @@
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>DC-HV2</t>
+          <t>DC-HTC</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>-4836039448</t>
+          <t>-4832751364</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
@@ -6198,11 +6198,11 @@
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr"/>
@@ -6218,12 +6218,12 @@
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>DC-NVK</t>
+          <t>DC-HV2</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>-4827088164</t>
+          <t>-4836039448</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
@@ -6232,7 +6232,7 @@
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
@@ -6252,12 +6252,12 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>DC-PPZ</t>
+          <t>DC-NVK</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>-4972623393</t>
+          <t>-4827088164</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="F171" s="2" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
@@ -6286,12 +6286,12 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>DC-PVB</t>
+          <t>DC-PPZ</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>-4724011528</t>
+          <t>-4972623393</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H172" s="3" t="inlineStr"/>
@@ -6320,12 +6320,12 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>DC-SCV</t>
+          <t>DC-PVB</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>-4922136877</t>
+          <t>-4724011528</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
@@ -6334,11 +6334,11 @@
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H173" s="3" t="inlineStr"/>
@@ -6354,12 +6354,12 @@
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>DC-THN</t>
+          <t>DC-SCV</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>-4982081891</t>
+          <t>-4922136877</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -6368,7 +6368,7 @@
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
@@ -6388,12 +6388,12 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>DMR - DC (Block C Diamond Riverside)</t>
+          <t>DC-THN</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>-4883865942</t>
+          <t>-4982081891</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -6422,25 +6422,25 @@
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>DS7 - DC (99 Đường Số 7)</t>
+          <t>DMR - DC (Block C Diamond Riverside)</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>-1002166724266</t>
+          <t>-4883865942</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H176" s="3" t="inlineStr"/>
@@ -6456,21 +6456,21 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>EH3- DC</t>
+          <t>DS7 - DC (99 Đường Số 7)</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>-4712243485</t>
+          <t>-1002166724266</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F177" s="2" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
@@ -6490,12 +6490,12 @@
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>GHA - DC (The Art Gia Hòa)</t>
+          <t>EH3- DC</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>-4125880558</t>
+          <t>-4712243485</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -6504,7 +6504,7 @@
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
@@ -6524,25 +6524,25 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>HHM - DC (165 Hoàng Hoa Thám)</t>
+          <t>GHA - DC (The Art Gia Hòa)</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>-1003822384320</t>
+          <t>-4125880558</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H179" s="3" t="inlineStr"/>
@@ -6563,15 +6563,17 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>-4612672037</t>
+          <t>-1003822384320</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr"/>
+          <t>Supergroup</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -6590,12 +6592,12 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>HLR - DC ( Block A Himlam Riverside Q7)</t>
+          <t>HHM - DC (165 Hoàng Hoa Thám)</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>-4943081238</t>
+          <t>-4612672037</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
@@ -6603,9 +6605,7 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F181" s="2" t="n">
-        <v>27</v>
-      </c>
+      <c r="F181" s="2" t="inlineStr"/>
       <c r="G181" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -6624,12 +6624,12 @@
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>HPD - DC (01-06 TMDV Him Lam Phú Đông)</t>
+          <t>HLR - DC ( Block A Himlam Riverside Q7)</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>-4820723298</t>
+          <t>-4943081238</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -6638,7 +6638,7 @@
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
@@ -6658,12 +6658,12 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>HTN - DC (17 Hồ Thị Nhung)</t>
+          <t>HPD - DC (01-06 TMDV Him Lam Phú Đông)</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>-4658447671</t>
+          <t>-4820723298</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
@@ -6672,7 +6672,7 @@
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
@@ -6692,12 +6692,12 @@
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>KDG - DC (10D Kỳ Đồng)</t>
+          <t>HTN - DC (17 Hồ Thị Nhung)</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>-4951125300</t>
+          <t>-4658447671</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -6706,11 +6706,11 @@
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H184" s="3" t="inlineStr"/>
@@ -6726,12 +6726,12 @@
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>LVH - DC (222 Lê Văn Thịnh)</t>
+          <t>KDG - DC (10D Kỳ Đồng)</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>-4614044179</t>
+          <t>-4951125300</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H185" s="3" t="inlineStr"/>
@@ -6760,12 +6760,12 @@
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>LVL - DC (166E Lê Văn Lương)</t>
+          <t>LVH - DC (222 Lê Văn Thịnh)</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>-884744948</t>
+          <t>-4614044179</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
@@ -6774,7 +6774,7 @@
         </is>
       </c>
       <c r="F186" s="2" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
@@ -6794,12 +6794,12 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>MZ2 - DC (A7-8 Valora Mizuki)</t>
+          <t>LVL - DC (166E Lê Văn Lương)</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>-4906931555</t>
+          <t>-884744948</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="F187" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
@@ -6828,12 +6828,12 @@
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>MZK - DC (TMDV2 Mizuki Park)</t>
+          <t>MZ2 - DC (A7-8 Valora Mizuki)</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>-4097174073</t>
+          <t>-4906931555</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
@@ -6842,7 +6842,7 @@
         </is>
       </c>
       <c r="F188" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
@@ -6862,12 +6862,12 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>NDH - DC (1426 Nguyễn Duy Trinh)</t>
+          <t>MZK - DC (TMDV2 Mizuki Park)</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>-4641160091</t>
+          <t>-4097174073</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
@@ -6876,7 +6876,7 @@
         </is>
       </c>
       <c r="F189" s="2" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
@@ -6896,12 +6896,12 @@
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>NTO - DC (108 Ngô Tất Tố)</t>
+          <t>NDH - DC (1426 Nguyễn Duy Trinh)</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>-4870440616</t>
+          <t>-4641160091</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
@@ -6910,11 +6910,11 @@
         </is>
       </c>
       <c r="F190" s="2" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>Mới thêm hôm nay</t>
+          <t>Đã có sẵn</t>
         </is>
       </c>
       <c r="H190" s="3" t="inlineStr"/>
@@ -6930,21 +6930,21 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>NTU - DC (46 Nguyễn Thị Tú)</t>
+          <t>NTO - DC (108 Ngô Tất Tố)</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>-1001929557412</t>
+          <t>-4870440616</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>Supergroup</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F191" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
@@ -6964,21 +6964,21 @@
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>NVD - DC (42 Nguyễn Văn Đậu)</t>
+          <t>NTU - DC (46 Nguyễn Thị Tú)</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>-4246704011</t>
+          <t>-1001929557412</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Supergroup</t>
         </is>
       </c>
       <c r="F192" s="2" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
@@ -6998,12 +6998,12 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Q7R - DC (Lô CD L1-12 Q7 Riverside Đào Trí)</t>
+          <t>NVD - DC (42 Nguyễn Văn Đậu)</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>-4610245241</t>
+          <t>-4246704011</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
@@ -7012,11 +7012,11 @@
         </is>
       </c>
       <c r="F193" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>Đã có sẵn</t>
+          <t>Mới thêm hôm nay</t>
         </is>
       </c>
       <c r="H193" s="3" t="inlineStr"/>
@@ -7032,12 +7032,12 @@
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>QHG_DC_ store</t>
+          <t>Q7R - DC (Lô CD L1-12 Q7 Riverside Đào Trí)</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>-4249658669</t>
+          <t>-4610245241</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
@@ -7046,7 +7046,7 @@
         </is>
       </c>
       <c r="F194" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
@@ -7066,12 +7066,12 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>RVS - DC (C0.01 Riverside Phú Mỹ Hưng)</t>
+          <t>QHG_DC_ store</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>-4928360925</t>
+          <t>-4249658669</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -7100,12 +7100,12 @@
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>VH2 - DC (S10.02 Vinhomes Grand Park)</t>
+          <t>RVS - DC (C0.01 Riverside Phú Mỹ Hưng)</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>-4077409269</t>
+          <t>-4928360925</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -7114,7 +7114,7 @@
         </is>
       </c>
       <c r="F196" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
@@ -7134,12 +7134,12 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>VH5 - DC (S03.05 Vinhomes Grand Park)</t>
+          <t>VH2 - DC (S10.02 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>-4971875234</t>
+          <t>-4077409269</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="F197" s="2" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
@@ -7168,12 +7168,12 @@
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>VH7 - DC (BS11 Vinhomes Grand Park)</t>
+          <t>VH5 - DC (S03.05 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>-4873359487</t>
+          <t>-4971875234</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -7182,7 +7182,7 @@
         </is>
       </c>
       <c r="F198" s="2" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
@@ -7202,12 +7202,12 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>VPC - DC (02 Nguyễn Thị Nhung)</t>
+          <t>VH7 - DC (BS11 Vinhomes Grand Park)</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>-4587582513</t>
+          <t>-4873359487</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
@@ -7215,7 +7215,9 @@
           <t>Group</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr"/>
+      <c r="F199" s="2" t="n">
+        <v>23</v>
+      </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
           <t>Đã có sẵn</t>
@@ -7239,23 +7241,55 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
+          <t>-4587582513</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr"/>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Đã có sẵn</t>
+        </is>
+      </c>
+      <c r="H200" s="3" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>VPC - DC (02 Nguyễn Thị Nhung)</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
           <t>-1003925120550</t>
         </is>
       </c>
-      <c r="E200" s="2" t="inlineStr">
+      <c r="E201" s="2" t="inlineStr">
         <is>
           <t>Supergroup</t>
         </is>
       </c>
-      <c r="F200" s="2" t="n">
+      <c r="F201" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="G200" s="2" t="inlineStr">
-        <is>
-          <t>Đã có sẵn</t>
-        </is>
-      </c>
-      <c r="H200" s="3" t="inlineStr"/>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>Đã có sẵn</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Cap nhat chat ID Jamila Khang Dien vao nhom DC va ghi nhan lich su spam 2 phieu chi tiet kho kho PT2003271, PT2003257
</commit_message>
<xml_diff>
--- a/Danh_Sach_Chat_ID_Nhom_DC.xlsx
+++ b/Danh_Sach_Chat_ID_Nhom_DC.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7425,6 +7425,44 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>JKD</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>DC - JKD( JAMILA Khang Điền )</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>-4207174927</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Đã có sẵn</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cap nhat A254 Phu Cuong Home vao Danh_Sach_Chat_ID_Nhom_DC va Tool Chi Tiet Kho Kho
</commit_message>
<xml_diff>
--- a/Danh_Sach_Chat_ID_Nhom_DC.xlsx
+++ b/Danh_Sach_Chat_ID_Nhom_DC.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7461,7 +7461,43 @@
           <t>Đã có sẵn</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>A254</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>DC - A254 (Phú Cường Home)</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>-1003932058795</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Supergroup</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Đã có sẵn</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>